<commit_message>
Surface INVALID_GEODATA import error, add Geo Data column to all templates
Only the "other countries" farmer import template exposed the Geo Data
column; Rwanda, Honduras, and the Spanish "otros países" template had no
header for it and no Read Me instructions, even though the backend reads
that column positionally for every company. Add the same column/width and
matching instruction line to those three templates, and render the new
backend INVALID_GEODATA validation error with a proper message instead of
falling through to "/".
</commit_message>
<xml_diff>
--- a/src/assets/farmer-import/Plantilla_listado_de_agricultores_Honduras_es.xlsx
+++ b/src/assets/farmer-import/Plantilla_listado_de_agricultores_Honduras_es.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pecea/Downloads/new import templates/"/>
     </mc:Choice>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t>List of farmers</t>
   </si>
@@ -123,11 +123,15 @@
   <si>
     <t>Dirección adicional (no aplica para Honduras)</t>
   </si>
+  <si>
+    <t>Datos geográficos (POLYGON((lat1 lon1, lat2 lon2,...)))</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1540,30 +1544,31 @@
   <dimension ref="A1:AM260"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="25.33203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="17" style="1" customWidth="1"/>
-    <col min="3" max="3" width="26.1640625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="23.33203125" style="1" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="22.33203125" style="1" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="19.83203125" style="1" hidden="1" customWidth="1"/>
-    <col min="7" max="10" width="19.83203125" style="1" customWidth="1"/>
-    <col min="11" max="15" width="19.83203125" style="1" hidden="1" customWidth="1"/>
-    <col min="16" max="17" width="29.1640625" style="1" customWidth="1"/>
-    <col min="18" max="18" width="17.1640625" style="1" customWidth="1"/>
-    <col min="19" max="19" width="19.6640625" style="1" customWidth="1"/>
-    <col min="20" max="20" width="18.33203125" style="1" customWidth="1"/>
-    <col min="21" max="21" width="26.5" style="1" customWidth="1"/>
-    <col min="22" max="24" width="18.33203125" style="1" customWidth="1"/>
-    <col min="25" max="25" width="30.83203125" style="1" customWidth="1"/>
-    <col min="26" max="26" width="31.6640625" style="1" customWidth="1"/>
-    <col min="27" max="28" width="18.33203125" style="1" customWidth="1"/>
-    <col min="29" max="29" width="20.5" style="1" customWidth="1"/>
-    <col min="30" max="30" width="26" style="1" customWidth="1"/>
-    <col min="31" max="31" width="21.1640625" style="1" customWidth="1"/>
-    <col min="32" max="32" width="25.5" style="1" customWidth="1"/>
-    <col min="33" max="33" width="22.6640625" style="1" customWidth="1"/>
-    <col min="34" max="40" width="8.6640625" style="1" customWidth="1"/>
-    <col min="41" max="16384" width="8.6640625" style="1"/>
+    <col min="35" max="40" customWidth="true" style="1" width="8.6640625"/>
+    <col min="1" max="1" customWidth="true" style="1" width="25.33203125"/>
+    <col min="2" max="2" customWidth="true" style="1" width="17.0"/>
+    <col min="3" max="3" customWidth="true" style="1" width="26.1640625"/>
+    <col min="4" max="4" customWidth="true" hidden="true" style="1" width="23.33203125"/>
+    <col min="5" max="5" customWidth="true" hidden="true" style="1" width="22.33203125"/>
+    <col min="6" max="6" customWidth="true" hidden="true" style="1" width="19.83203125"/>
+    <col min="7" max="10" customWidth="true" style="1" width="19.83203125"/>
+    <col min="11" max="15" customWidth="true" hidden="true" style="1" width="19.83203125"/>
+    <col min="16" max="17" customWidth="true" style="1" width="29.1640625"/>
+    <col min="18" max="18" customWidth="true" style="1" width="17.1640625"/>
+    <col min="19" max="19" customWidth="true" style="1" width="19.6640625"/>
+    <col min="20" max="20" customWidth="true" style="1" width="18.33203125"/>
+    <col min="21" max="21" customWidth="true" style="1" width="26.5"/>
+    <col min="22" max="24" customWidth="true" style="1" width="18.33203125"/>
+    <col min="25" max="25" customWidth="true" style="1" width="30.83203125"/>
+    <col min="26" max="26" customWidth="true" style="1" width="31.6640625"/>
+    <col min="27" max="28" customWidth="true" style="1" width="18.33203125"/>
+    <col min="29" max="29" customWidth="true" style="1" width="20.5"/>
+    <col min="30" max="30" customWidth="true" style="1" width="26.0"/>
+    <col min="31" max="31" customWidth="true" style="1" width="21.1640625"/>
+    <col min="32" max="32" customWidth="true" style="1" width="25.5"/>
+    <col min="33" max="33" customWidth="true" style="1" width="22.6640625"/>
+    <col min="34" max="34" customWidth="true" style="1" width="29.5703125"/>
+    <col min="41" max="16384" style="1" width="8.6640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -1832,7 +1837,9 @@
       <c r="AG5" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="AH5" s="9"/>
+      <c r="AH5" s="24" t="s">
+        <v>34</v>
+      </c>
       <c r="AI5" s="3"/>
       <c r="AJ5" s="3"/>
       <c r="AK5" s="3"/>

</xml_diff>

<commit_message>
add geoID to import template
</commit_message>
<xml_diff>
--- a/src/assets/farmer-import/Plantilla_listado_de_agricultores_Honduras_es.xlsx
+++ b/src/assets/farmer-import/Plantilla_listado_de_agricultores_Honduras_es.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>List of farmers</t>
   </si>
@@ -125,6 +125,12 @@
   </si>
   <si>
     <t>Datos geográficos (POLYGON((lat1 lon1, lat2 lon2,...)))</t>
+  </si>
+  <si>
+    <t>Datos geográficos (POLYGON((lat1 lon1, lat2 lon2,...)), POINT(lat lon), GeoJSON, geoshape de ODK/Kobo "lat lon alt prec;...", o P1(...)P2(...) para varias parcelas)</t>
+  </si>
+  <si>
+    <t>GeoID (FAO) - identificador del límite de la parcela en el registro GeoID de la FAO</t>
   </si>
 </sst>
 </file>
@@ -1544,7 +1550,7 @@
   <dimension ref="A1:AM260"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="35" max="40" customWidth="true" style="1" width="8.6640625"/>
+    <col min="36" max="40" customWidth="true" style="1" width="8.6640625"/>
     <col min="1" max="1" customWidth="true" style="1" width="25.33203125"/>
     <col min="2" max="2" customWidth="true" style="1" width="17.0"/>
     <col min="3" max="3" customWidth="true" style="1" width="26.1640625"/>
@@ -1568,6 +1574,7 @@
     <col min="32" max="32" customWidth="true" style="1" width="25.5"/>
     <col min="33" max="33" customWidth="true" style="1" width="22.6640625"/>
     <col min="34" max="34" customWidth="true" style="1" width="29.5703125"/>
+    <col min="35" max="35" customWidth="true" style="1" width="29.5703125"/>
     <col min="41" max="16384" style="1" width="8.6640625"/>
   </cols>
   <sheetData>
@@ -1838,9 +1845,11 @@
         <v>29</v>
       </c>
       <c r="AH5" s="24" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
-      <c r="AI5" s="3"/>
+      <c r="AI5" s="24" t="s">
+        <v>36</v>
+      </c>
       <c r="AJ5" s="3"/>
       <c r="AK5" s="3"/>
       <c r="AL5" s="3"/>

</xml_diff>